<commit_message>
fix isDialogDisplayed => done
</commit_message>
<xml_diff>
--- a/ExportExcel/Add Academic Degrees Test.xlsx
+++ b/ExportExcel/Add Academic Degrees Test.xlsx
@@ -41,37 +41,37 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>7323 ms</t>
+    <t>6625 ms</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
+    <t>testAddADMErrorWithDuplicateID</t>
+  </si>
+  <si>
+    <t>TC_AddADM_02</t>
+  </si>
+  <si>
+    <t>8221 ms</t>
+  </si>
+  <si>
     <t>testAddADMErrorWithDataMaxLength</t>
   </si>
   <si>
-    <t>TC_AddADM_02</t>
-  </si>
-  <si>
-    <t>7758 ms</t>
+    <t>TC_AddADM_03</t>
+  </si>
+  <si>
+    <t>8287 ms</t>
   </si>
   <si>
     <t>testAddADMErrorWithDataEmpty</t>
   </si>
   <si>
-    <t>TC_AddADM_03</t>
-  </si>
-  <si>
-    <t>8483 ms</t>
-  </si>
-  <si>
-    <t>testAddADMErrorWithDuplicateID</t>
-  </si>
-  <si>
     <t>TC_AddADM_04</t>
   </si>
   <si>
-    <t>5657 ms</t>
+    <t>8914 ms</t>
   </si>
   <si>
     <t>testAddADMErrorWithInvalidFormat</t>
@@ -80,7 +80,7 @@
     <t>TC_AddADM_05</t>
   </si>
   <si>
-    <t>8345 ms</t>
+    <t>8380 ms</t>
   </si>
   <si>
     <t>testAddADMErrorWithDataMinLength</t>
@@ -89,7 +89,7 @@
     <t>TC_AddADM_06</t>
   </si>
   <si>
-    <t>5336 ms</t>
+    <t>5377 ms</t>
   </si>
 </sst>
 </file>

</xml_diff>